<commit_message>
Intrastat-App: Firmenauswahl (KST/KSPC), UI-Politur der Prüfansicht und Doku
Erweitert die App um eine Firmenauswahl (Kläger Spraying Technology /
Kläger Performance Components) mit eigenem Farbschema, eigenen
Gewichtslisten je Firma und firmenspezifischen Export-Dateinamen.
Überarbeitet die Prüfansicht (Ein-/Ausklappen und Ein-/Ausblenden von
Rechnungen, Suche, Sortierung), verfeinert das KI-Auslesen von
Ausgangs- und Eingangsrechnungen (Adress-/Gewichts-Erkennung,
Datumsauflösung) und aktualisiert Dokumentation sowie Testsuite
entsprechend. Nicht mehr benötigte Assets (lokale PDF-Verarbeitung)
wurden entfernt, da Claude die alleinige Quelle der Rechnungsdaten ist.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/Mustertabelle.xlsx
+++ b/src/assets/Mustertabelle.xlsx
@@ -1,21 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wisseborn\Desktop\Neuer Ordner\Intrastat\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A913C32-E727-481E-BECC-440F3E51B8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Warenbewegung" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Warenbewegung" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -25,63 +16,68 @@
     <t>Richtung</t>
   </si>
   <si>
-    <t>E oder V</t>
-  </si>
-  <si>
     <t>Bezugsmonat</t>
   </si>
   <si>
     <t>Art des Geschäftes</t>
   </si>
   <si>
-    <t>Besondere Maßeinheit</t>
-  </si>
-  <si>
-    <t>01, 02….</t>
-  </si>
-  <si>
-    <t>Statistischer Wert in vollen €</t>
-  </si>
-  <si>
     <t>Verkehrszweig</t>
   </si>
   <si>
-    <t>Rechnungsbetrag in vollen €</t>
-  </si>
-  <si>
-    <t>Warennummer 8-stellig</t>
-  </si>
-  <si>
-    <t>Eigenmasse
-in vollen kg</t>
-  </si>
-  <si>
-    <t>Ursprungsland</t>
-  </si>
-  <si>
-    <t>USt-IdNr. des Warenempfängers
-(Nur Versendung)</t>
-  </si>
-  <si>
-    <t>Warenbezeichnung (max. 105 Zeichen, Angabe freiwillig)</t>
-  </si>
-  <si>
-    <t>Versendungs-
+    <t xml:space="preserve">Versendungs-
 mitgliedstaat
 nur Eingang</t>
   </si>
   <si>
-    <t>Bestimmungs-
+    <t xml:space="preserve">Bestimmungs-
 mitgliedstaat
 nur Versendung</t>
   </si>
   <si>
-    <t>Bestimmungs-
-bundesland nur Eingang</t>
-  </si>
-  <si>
-    <t>Ursprungs-
-bundesland nur Versendung</t>
+    <t xml:space="preserve">Bestimmungs-
+bundesland
+nur Eingang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ursprungs-
+bundesland
+nur Versendung</t>
+  </si>
+  <si>
+    <t>Ursprungsland</t>
+  </si>
+  <si>
+    <t>Warennummer 8-stellig</t>
+  </si>
+  <si>
+    <t>Warenbezeichnung (max. 105 Zeichen, Angabe freiwillig)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigenmasse
+in vollen kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Besondere
+Maßeinheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechnungsbetrag
+in vollen €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistischer Wert
+in vollen €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt-IdNr. des Warenempfängers
+(Nur Versendung)</t>
+  </si>
+  <si>
+    <t>E oder V</t>
+  </si>
+  <si>
+    <t>01, 02….</t>
   </si>
   <si>
     <t>Definitionen zu den Merkmalen: Siehe entsprechenden Anfangsbuchstaben im Stichwortverzeichnis (https://erhebungsportal.estatistik.de/Erhebungsportal/informationen/stichwortverzeichnis-4279)</t>
@@ -90,38 +86,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="00"/>
-    <numFmt numFmtId="165" formatCode="00000000"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
       <color indexed="10"/>
-      <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
     </font>
     <font>
       <u/>
+      <color indexed="12"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color indexed="12"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
     </font>
   </fonts>
   <fills count="2">
@@ -141,38 +133,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
+  </cellStyleXfs>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -188,9 +168,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -228,7 +208,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -300,7 +280,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -332,20 +312,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -467,125 +443,147 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="20.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="11.42578125" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="26.28515625" customWidth="1"/>
     <col min="4" max="4" width="14.140625" customWidth="1"/>
-    <col min="5" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" customWidth="1"/>
-    <col min="15" max="15" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="30.28515625" customWidth="1"/>
+    <col min="12" max="15" width="20.7109375" customWidth="1"/>
+    <col min="16" max="16" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" ht="36" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="80.1" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="3" t="s">
+    </row>
+    <row r="2" ht="20.1" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="C2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
     </row>
-    <row r="2" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="J3" s="7"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-    </row>
-    <row r="5" spans="1:16" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="siehe Stichwortverzeichnis" xr:uid="{610F5D12-740E-436D-8D4B-71A933EFB7AA}"/>
-    <hyperlink ref="C2:K2" r:id="rId2" display="Definitionen zu den Merkmalen: siehe entsprechenden Anfangbuchstaben im Stichwortverzeichnis (https://erhebungsportal.estatistik.de/Erhebungsportal/informationen/stichwortverzeichnis-4279)" xr:uid="{A9EB3D2C-0788-4230-8DCB-7A54FEE4E124}"/>
+    <hyperlink ref="C2" r:id="rId1"/>
   </hyperlinks>
-  <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
-  <headerFooter alignWithMargins="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>